<commit_message>
Datos y alertas 2026-07-08
</commit_message>
<xml_diff>
--- a/alertas/alertas_2026-07-07.xlsx
+++ b/alertas/alertas_2026-07-07.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="43">
   <si>
     <t>Fecha</t>
   </si>
@@ -31,25 +31,31 @@
     <t>Unidad</t>
   </si>
   <si>
+    <t>07/07/2026 04:14</t>
+  </si>
+  <si>
+    <t>heladera BM muestras</t>
+  </si>
+  <si>
+    <t>ambiente</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> °C</t>
+  </si>
+  <si>
+    <t>07/07/2026 04:10</t>
+  </si>
+  <si>
+    <t>heladera BM reactivos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ambiente </t>
+  </si>
+  <si>
     <t>07/07/2026 03:59</t>
   </si>
   <si>
-    <t>heladera BM muestras</t>
-  </si>
-  <si>
-    <t>ambiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> °C</t>
-  </si>
-  <si>
     <t>07/07/2026 03:54</t>
-  </si>
-  <si>
-    <t>heladera BM reactivos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ambiente </t>
   </si>
   <si>
     <t>07/07/2026 03:44</t>
@@ -510,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="20" customWidth="1"/>
@@ -648,10 +654,10 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E8">
-        <v>-15</v>
+        <v>26</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -659,13 +665,13 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E9">
         <v>26</v>
@@ -676,16 +682,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
         <v>20</v>
       </c>
-      <c r="C10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
       <c r="E10">
-        <v>26</v>
+        <v>-15</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
@@ -699,10 +705,10 @@
         <v>7</v>
       </c>
       <c r="D11" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E11">
-        <v>-15</v>
+        <v>26</v>
       </c>
       <c r="F11" t="s">
         <v>9</v>
@@ -713,10 +719,10 @@
         <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E12">
         <v>26</v>
@@ -730,13 +736,13 @@
         <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E13">
-        <v>26</v>
+        <v>-15</v>
       </c>
       <c r="F13" t="s">
         <v>9</v>
@@ -832,21 +838,21 @@
         <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E19">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F19" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C20" t="s">
         <v>7</v>
@@ -863,19 +869,19 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" t="s">
+        <v>33</v>
+      </c>
+      <c r="E21">
+        <v>10</v>
+      </c>
+      <c r="F21" t="s">
         <v>34</v>
-      </c>
-      <c r="C21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21">
-        <v>26</v>
-      </c>
-      <c r="F21" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -900,10 +906,10 @@
         <v>36</v>
       </c>
       <c r="C23" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D23" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E23">
         <v>26</v>
@@ -917,13 +923,13 @@
         <v>37</v>
       </c>
       <c r="C24" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E24">
-        <v>-15</v>
+        <v>26</v>
       </c>
       <c r="F24" t="s">
         <v>9</v>
@@ -934,13 +940,13 @@
         <v>38</v>
       </c>
       <c r="C25" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="E25">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="F25" t="s">
         <v>9</v>
@@ -948,18 +954,52 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C26" t="s">
         <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E26">
         <v>-15</v>
       </c>
       <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" t="s">
+        <v>33</v>
+      </c>
+      <c r="E27">
+        <v>8</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28">
+        <v>-15</v>
+      </c>
+      <c r="F28" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>